<commit_message>
Replace LTV standard/FTB/BTL columns with FTB/OOO, SSB/BTL, and other limits.
The old "standard" cap mixed unrelated percentages across country taxonomies. Gold, extraction, dashboard, and Supabase now group borrower/use (and leftover differentiations) instead.
</commit_message>
<xml_diff>
--- a/reports/downloads/capital_overall_buffers.xlsx
+++ b/reports/downloads/capital_overall_buffers.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,41 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ISO2</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>CCoB</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>CCyB</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>GSII/O-SII</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>SyRB</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>sSyRB</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -469,113 +481,113 @@
         <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IS</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2.5</v>
       </c>
       <c r="C3" t="n">
-        <v>2.5</v>
+        <v>1.25</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>8</v>
+        <v>11.25</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>IS</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>2.5</v>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D4" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CZ</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>2.5</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="7">
@@ -594,226 +606,226 @@
         <v>2</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>6.5</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EE</t>
+          <t>BG</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>2.5</v>
       </c>
       <c r="C8" t="n">
-        <v>1.5</v>
+        <v>2.25</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>2.5</v>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>2.5</v>
       </c>
       <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E10" t="n">
         <v>1.5</v>
       </c>
-      <c r="D10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CY</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>2.5</v>
       </c>
       <c r="C11" t="n">
-        <v>1.5</v>
+        <v>0.75</v>
       </c>
       <c r="D11" t="n">
-        <v>1.9375</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>5.9375</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BG</t>
+          <t>EE</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>2.5</v>
       </c>
       <c r="C12" t="n">
-        <v>2.25</v>
+        <v>1.5</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>5.75</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>2.5</v>
       </c>
       <c r="C13" t="n">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G13" t="n">
-        <v>5.75</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HU</t>
+          <t>LI</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>2.5</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IE</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>2.5</v>
       </c>
       <c r="C15" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>5.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LV</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>2.5</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="D16" t="n">
         <v>2</v>
@@ -822,91 +834,91 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G16" t="n">
-        <v>5.5</v>
+        <v>7.75</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>CZ</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>2.5</v>
       </c>
       <c r="C17" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D17" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>5.5</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>2.5</v>
       </c>
       <c r="C18" t="n">
-        <v>1.25</v>
+        <v>0.75</v>
       </c>
       <c r="D18" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" t="n">
-        <v>5.25</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>SK</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>2.5</v>
       </c>
       <c r="C19" t="n">
-        <v>0.75</v>
+        <v>1.5</v>
       </c>
       <c r="D19" t="n">
         <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>5.25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FI</t>
+          <t>AT</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -916,32 +928,32 @@
         <v>0</v>
       </c>
       <c r="D20" t="n">
-        <v>2.5</v>
+        <v>1.75</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>5</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>CY</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>2.5</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D21" t="n">
-        <v>1.5</v>
+        <v>2.25</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -950,57 +962,57 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>5</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>FI</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>2.5</v>
       </c>
       <c r="C22" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>2.5</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
-        <v>1.25</v>
+        <v>2</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>4.75</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
@@ -1022,23 +1034,23 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>4.75</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LI</t>
+          <t>HU</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>2.5</v>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
         <v>2</v>
@@ -1050,23 +1062,23 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>IE</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>2.5</v>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
@@ -1075,23 +1087,23 @@
         <v>0</v>
       </c>
       <c r="G26" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AT</t>
+          <t>LV</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>2.5</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -1100,20 +1112,20 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>4.25</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GR</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>2.5</v>
       </c>
       <c r="C28" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
         <v>1.25</v>
@@ -1125,48 +1137,48 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>4.25</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>2.5</v>
       </c>
       <c r="C29" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>4.25</v>
+        <v>4.75</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>GR</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2.5</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D30" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -1175,7 +1187,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="31">
@@ -1201,6 +1213,31 @@
       </c>
       <c r="G31" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>